<commit_message>
Make Kobo KPI choices upload compatible
</commit_message>
<xml_diff>
--- a/kobo_forms/PMS_GMC_Formulaire_1_Referentiel_KPI_Formules_2026.xlsx
+++ b/kobo_forms/PMS_GMC_Formulaire_1_Referentiel_KPI_Formules_2026.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R9694f3ab8f194ae4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R647f4d2c621a4639"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rfa78f26329904d6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R57d815127e5044df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rfed946838f4d4c6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R0dd287f4f9444569"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>